<commit_message>
Corrected the excel files
</commit_message>
<xml_diff>
--- a/data/Heat map 1.xlsx
+++ b/data/Heat map 1.xlsx
@@ -1,197 +1,340 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BB90A00-C62E-4F71-AE5E-4EA14CC71862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="30195" yWindow="1395" windowWidth="27000" windowHeight="15735" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Res, Cap, Product" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Res, Cap, Product" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_Hlk200085589" localSheetId="0">'Res, Cap, Product'!#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Res, Cap, Product'!$B$1:$P$19</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
+  <si>
+    <t>KPI by Nr.</t>
+  </si>
+  <si>
+    <t>Research Outputs</t>
+  </si>
+  <si>
+    <t>Training and Capacity Building</t>
+  </si>
+  <si>
+    <t>Product Development</t>
+  </si>
+  <si>
+    <t>Thomson indexed publications</t>
+  </si>
+  <si>
+    <t>Publications per IRS</t>
+  </si>
+  <si>
+    <t>High impact publications</t>
+  </si>
+  <si>
+    <t>PhD and MsC  students enrolled</t>
+  </si>
+  <si>
+    <t>PhD and MsC  theses completed</t>
+  </si>
+  <si>
+    <t>Stakeholders trained on innovations</t>
+  </si>
+  <si>
+    <t>Training to NARES by IITA Scientists</t>
+  </si>
+  <si>
+    <t>Varieties released</t>
+  </si>
+  <si>
+    <t>Genetic gain rate</t>
+  </si>
+  <si>
+    <t>Crop Trust compliance rate</t>
+  </si>
+  <si>
+    <t>Innovations in e-Catalogue</t>
+  </si>
+  <si>
+    <t>Innovations taken on by scaling partners</t>
+  </si>
+  <si>
+    <t>GI</t>
+  </si>
+  <si>
+    <t>Biotech</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Breeding</t>
+  </si>
+  <si>
+    <t>Genebanks</t>
+  </si>
+  <si>
+    <t>Seed System</t>
+  </si>
+  <si>
+    <t>RAFS</t>
+  </si>
+  <si>
+    <t>Plant Health</t>
+  </si>
+  <si>
+    <t>Farming Systems Agronomy</t>
+  </si>
+  <si>
+    <t>NRM</t>
+  </si>
+  <si>
+    <t>Mechanization</t>
+  </si>
+  <si>
+    <t>ST</t>
+  </si>
+  <si>
+    <t>FIAS</t>
+  </si>
+  <si>
+    <t>GeYSI</t>
+  </si>
+  <si>
+    <t>RCA</t>
+  </si>
+  <si>
+    <t>Nutrition</t>
+  </si>
+  <si>
+    <t>VCMA</t>
+  </si>
+  <si>
+    <t>2025 Actual Values</t>
+  </si>
+  <si>
+    <t>Annual Target</t>
+  </si>
+  <si>
+    <t>Per Program Target (target/13)</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It looks like the colorscheme is not consistently applied everywhere </t>
+  </si>
+  <si>
+    <t>(e.g., see the different versions of red in cells G4 and H4)?</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="5">
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="18"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="14"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF00B0F0"/>
-      <sz val="14"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="14"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="14"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="9"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="9"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF00B050"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF00B050"/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF00B050"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF0070C0"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="8"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="9"/>
     </font>
     <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <color rgb="FFFF0000"/>
-      <sz val="14"/>
     </font>
     <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="14"/>
     </font>
     <font>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="16"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.09997863704336681"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -574,251 +717,192 @@
     </border>
   </borders>
   <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="75">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1138,1016 +1222,866 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="4.21875" customWidth="1" min="1" max="1"/>
-    <col width="3.21875" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="24.88671875" bestFit="1" customWidth="1" style="59" min="3" max="3"/>
-    <col width="8" customWidth="1" style="2" min="4" max="4"/>
-    <col width="8" customWidth="1" style="57" min="5" max="5"/>
-    <col width="8" customWidth="1" style="58" min="6" max="6"/>
-    <col width="8" customWidth="1" style="2" min="7" max="15"/>
-    <col width="9.33203125" customWidth="1" style="2" min="16" max="16"/>
-    <col width="8.21875" customWidth="1" style="3" min="17" max="21"/>
+    <col min="1" max="1" width="4.21875" customWidth="1"/>
+    <col min="2" max="2" width="3.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.88671875" style="59" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="2" customWidth="1"/>
+    <col min="5" max="5" width="8" style="57" customWidth="1"/>
+    <col min="6" max="6" width="8" style="58" customWidth="1"/>
+    <col min="7" max="15" width="8" style="2" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" style="2" customWidth="1"/>
+    <col min="17" max="21" width="8.21875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" thickBot="1">
-      <c r="A1" s="1" t="n"/>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="72" t="inlineStr">
-        <is>
-          <t>KPI by Nr.</t>
-        </is>
-      </c>
-      <c r="D1" s="73" t="n"/>
-      <c r="E1" s="73" t="n"/>
-      <c r="F1" s="73" t="n"/>
-      <c r="G1" s="73" t="n"/>
-      <c r="H1" s="73" t="n"/>
-      <c r="I1" s="73" t="n"/>
-      <c r="J1" s="73" t="n"/>
-      <c r="K1" s="73" t="n"/>
-      <c r="L1" s="73" t="n"/>
-      <c r="M1" s="73" t="n"/>
-      <c r="N1" s="73" t="n"/>
-      <c r="O1" s="74" t="n"/>
+    <row r="1" spans="1:21" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="74"/>
     </row>
-    <row r="2" ht="18.6" customFormat="1" customHeight="1" s="8" thickBot="1">
-      <c r="A2" s="4" t="n"/>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="63" t="inlineStr">
-        <is>
-          <t>Research Outputs</t>
-        </is>
-      </c>
-      <c r="E2" s="64" t="n"/>
-      <c r="F2" s="65" t="n"/>
-      <c r="G2" s="69" t="inlineStr">
-        <is>
-          <t>Training and Capacity Building</t>
-        </is>
-      </c>
-      <c r="H2" s="64" t="n"/>
-      <c r="I2" s="64" t="n"/>
-      <c r="J2" s="65" t="n"/>
-      <c r="K2" s="69" t="inlineStr">
-        <is>
-          <t>Product Development</t>
-        </is>
-      </c>
-      <c r="L2" s="64" t="n"/>
-      <c r="M2" s="64" t="n"/>
-      <c r="N2" s="64" t="n"/>
-      <c r="O2" s="65" t="n"/>
-      <c r="P2" s="6" t="n"/>
-      <c r="Q2" s="7" t="n"/>
-      <c r="R2" s="7" t="n"/>
-      <c r="S2" s="7" t="n"/>
-      <c r="T2" s="7" t="n"/>
-      <c r="U2" s="7" t="n"/>
+    <row r="2" spans="1:21" s="8" customFormat="1" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="63" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="64"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="69" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="69" t="s">
+        <v>3</v>
+      </c>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="64"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="7"/>
     </row>
-    <row r="3" ht="143.55" customFormat="1" customHeight="1" s="17" thickBot="1">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="11" t="inlineStr">
-        <is>
-          <t>Thomson indexed publications</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>Publications per IRS</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>High impact publications</t>
-        </is>
-      </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>PhD and MsC  students enrolled</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>PhD and MsC  theses completed</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>Stakeholders trained on innovations</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>Training to NARES by IITA Scientists</t>
-        </is>
-      </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>Varieties released</t>
-        </is>
-      </c>
-      <c r="L3" s="14" t="inlineStr">
-        <is>
-          <t>Genetic gain rate</t>
-        </is>
-      </c>
-      <c r="M3" s="14" t="inlineStr">
-        <is>
-          <t>Crop Trust compliance rate</t>
-        </is>
-      </c>
-      <c r="N3" s="12" t="inlineStr">
-        <is>
-          <t>Innovations in e-Catalogue</t>
-        </is>
-      </c>
-      <c r="O3" s="13" t="inlineStr">
-        <is>
-          <t>Innovations taken on by scaling partners</t>
-        </is>
-      </c>
-      <c r="P3" s="15" t="n"/>
-      <c r="Q3" s="16" t="n"/>
-      <c r="R3" s="16" t="n"/>
-      <c r="S3" s="16" t="n"/>
-      <c r="T3" s="16" t="n"/>
-      <c r="U3" s="16" t="n"/>
+    <row r="3" spans="1:21" s="17" customFormat="1" ht="143.55000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="L3" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="O3" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
     </row>
-    <row r="4" ht="15.6" customHeight="1">
-      <c r="A4" s="1" t="n"/>
-      <c r="B4" s="66" t="inlineStr">
-        <is>
-          <t>GI</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>Biotech</t>
-        </is>
-      </c>
-      <c r="D4" s="19" t="n">
+    <row r="4" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1"/>
+      <c r="B4" s="66" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="19">
         <v>21.95</v>
       </c>
-      <c r="E4" s="20" t="n">
-        <v>3.135714285714286</v>
-      </c>
-      <c r="F4" s="21" t="n">
+      <c r="E4" s="20">
+        <v>3.1357142857142861</v>
+      </c>
+      <c r="F4" s="21">
         <v>1</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="19">
         <v>1</v>
       </c>
-      <c r="H4" s="22" t="n">
+      <c r="H4" s="22">
         <v>1</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="22">
         <v>68</v>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="J4" s="23">
         <v>184</v>
       </c>
-      <c r="K4" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L4" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M4" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N4" s="22" t="n">
+      <c r="K4" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="N4" s="22">
         <v>1</v>
       </c>
-      <c r="O4" s="23" t="n">
+      <c r="O4" s="23">
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="15.6" customHeight="1">
-      <c r="A5" s="1" t="n"/>
-      <c r="B5" s="67" t="n"/>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>Breeding</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="n">
+    <row r="5" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="67"/>
+      <c r="C5" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="25">
         <v>51.45</v>
       </c>
-      <c r="E5" s="26" t="n">
-        <v>2.236956521739131</v>
-      </c>
-      <c r="F5" s="27" t="n">
+      <c r="E5" s="26">
+        <v>2.2369565217391312</v>
+      </c>
+      <c r="F5" s="27">
         <v>0</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="25">
         <v>24</v>
       </c>
-      <c r="H5" s="28" t="n">
+      <c r="H5" s="28">
         <v>28</v>
       </c>
-      <c r="I5" s="28" t="n">
+      <c r="I5" s="28">
         <v>108</v>
       </c>
-      <c r="J5" s="29" t="n">
+      <c r="J5" s="29">
         <v>214</v>
       </c>
-      <c r="K5" s="25" t="n">
+      <c r="K5" s="25">
         <v>15</v>
       </c>
-      <c r="L5" s="30" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="M5" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N5" s="28" t="n">
+      <c r="L5" s="30">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="M5" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="N5" s="28">
         <v>8</v>
       </c>
-      <c r="O5" s="29" t="n">
+      <c r="O5" s="29">
         <v>5</v>
       </c>
     </row>
-    <row r="6" ht="15.6" customHeight="1">
-      <c r="A6" s="1" t="n"/>
-      <c r="B6" s="67" t="n"/>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>Genebanks</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="n">
+    <row r="6" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="1"/>
+      <c r="B6" s="67"/>
+      <c r="C6" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="25">
         <v>5</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="26">
         <v>1.25</v>
       </c>
-      <c r="F6" s="27" t="n">
+      <c r="F6" s="27">
         <v>0</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="25">
         <v>26</v>
       </c>
-      <c r="H6" s="28" t="n">
+      <c r="H6" s="28">
         <v>19</v>
       </c>
-      <c r="I6" s="28" t="n">
+      <c r="I6" s="28">
         <v>5</v>
       </c>
-      <c r="J6" s="29" t="n">
+      <c r="J6" s="29">
         <v>113</v>
       </c>
-      <c r="K6" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L6" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M6" s="31" t="n">
+      <c r="K6" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M6" s="31">
         <v>1</v>
       </c>
-      <c r="N6" s="28" t="n">
+      <c r="N6" s="28">
         <v>0</v>
       </c>
-      <c r="O6" s="29" t="n">
+      <c r="O6" s="29">
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A7" s="1" t="n"/>
-      <c r="B7" s="68" t="n"/>
-      <c r="C7" s="32" t="inlineStr">
-        <is>
-          <t>Seed System</t>
-        </is>
-      </c>
-      <c r="D7" s="33" t="n">
+    <row r="7" spans="1:21" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1"/>
+      <c r="B7" s="68"/>
+      <c r="C7" s="32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="33">
         <v>15.4</v>
       </c>
-      <c r="E7" s="34" t="n">
-        <v>1.026666666666667</v>
-      </c>
-      <c r="F7" s="35" t="n">
+      <c r="E7" s="34">
+        <v>1.0266666666666671</v>
+      </c>
+      <c r="F7" s="35">
         <v>0</v>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="33">
         <v>5</v>
       </c>
-      <c r="H7" s="36" t="n">
+      <c r="H7" s="36">
         <v>7</v>
       </c>
-      <c r="I7" s="36" t="n">
+      <c r="I7" s="36">
         <v>2247</v>
       </c>
-      <c r="J7" s="37" t="n">
+      <c r="J7" s="37">
         <v>309</v>
       </c>
-      <c r="K7" s="33" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L7" s="36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M7" s="36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N7" s="36" t="n">
+      <c r="K7" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="L7" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="M7" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="N7" s="36">
         <v>17</v>
       </c>
-      <c r="O7" s="37" t="n">
+      <c r="O7" s="37">
         <v>2</v>
       </c>
     </row>
-    <row r="8" ht="15.6" customHeight="1">
-      <c r="A8" s="1" t="n"/>
-      <c r="B8" s="66" t="inlineStr">
-        <is>
-          <t>RAFS</t>
-        </is>
-      </c>
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>Plant Health</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="n">
+    <row r="8" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="66" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="19">
         <v>41.45</v>
       </c>
-      <c r="E8" s="20" t="n">
-        <v>3.454166666666667</v>
-      </c>
-      <c r="F8" s="21" t="n">
+      <c r="E8" s="20">
+        <v>3.4541666666666671</v>
+      </c>
+      <c r="F8" s="21">
         <v>1</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="19">
         <v>9</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="22">
         <v>9</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="I8" s="22">
         <v>102</v>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="J8" s="23">
         <v>10</v>
       </c>
-      <c r="K8" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L8" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M8" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N8" s="22" t="n">
+      <c r="K8" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L8" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="M8" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="N8" s="22">
         <v>6</v>
       </c>
-      <c r="O8" s="23" t="n">
+      <c r="O8" s="23">
         <v>2</v>
       </c>
     </row>
-    <row r="9" ht="15.6" customHeight="1">
-      <c r="A9" s="1" t="n"/>
-      <c r="B9" s="67" t="n"/>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>Farming Systems Agronomy</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="n">
+    <row r="9" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="67"/>
+      <c r="C9" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="25">
         <v>20.87</v>
       </c>
-      <c r="E9" s="26" t="n">
-        <v>1.0435</v>
-      </c>
-      <c r="F9" s="27" t="n">
+      <c r="E9" s="26">
+        <v>1.0435000000000001</v>
+      </c>
+      <c r="F9" s="27">
         <v>1</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="25">
         <v>22</v>
       </c>
-      <c r="H9" s="28" t="n">
+      <c r="H9" s="28">
         <v>14</v>
       </c>
-      <c r="I9" s="28" t="n">
+      <c r="I9" s="28">
         <v>3185</v>
       </c>
-      <c r="J9" s="29" t="n">
+      <c r="J9" s="29">
         <v>233</v>
       </c>
-      <c r="K9" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L9" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M9" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N9" s="28" t="n">
+      <c r="K9" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L9" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M9" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="N9" s="28">
         <v>1</v>
       </c>
-      <c r="O9" s="29" t="n">
+      <c r="O9" s="29">
         <v>9</v>
       </c>
     </row>
-    <row r="10" ht="15.6" customHeight="1">
-      <c r="A10" s="1" t="n"/>
-      <c r="B10" s="67" t="n"/>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>NRM</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="n">
+    <row r="10" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="67"/>
+      <c r="C10" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="25">
         <v>15.5</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="26">
         <v>2.214285714285714</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="27">
         <v>2</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="G10" s="25">
         <v>7</v>
       </c>
-      <c r="H10" s="28" t="n">
+      <c r="H10" s="28">
         <v>3</v>
       </c>
-      <c r="I10" s="28" t="n">
+      <c r="I10" s="28">
         <v>3754</v>
       </c>
-      <c r="J10" s="29" t="n">
+      <c r="J10" s="29">
         <v>20</v>
       </c>
-      <c r="K10" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L10" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M10" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N10" s="28" t="n">
+      <c r="K10" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L10" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M10" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="28">
         <v>10</v>
       </c>
-      <c r="O10" s="29" t="n">
+      <c r="O10" s="29">
         <v>2</v>
       </c>
     </row>
-    <row r="11" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A11" s="1" t="n"/>
-      <c r="B11" s="68" t="n"/>
-      <c r="C11" s="32" t="inlineStr">
-        <is>
-          <t>Mechanization</t>
-        </is>
-      </c>
-      <c r="D11" s="33" t="n">
+    <row r="11" spans="1:21" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11" s="68"/>
+      <c r="C11" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="33">
         <v>0</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="34">
         <v>0</v>
       </c>
-      <c r="F11" s="35" t="n">
+      <c r="F11" s="35">
         <v>0</v>
       </c>
-      <c r="G11" s="33" t="n">
+      <c r="G11" s="33">
         <v>2</v>
       </c>
-      <c r="H11" s="36" t="n">
+      <c r="H11" s="36">
         <v>1</v>
       </c>
-      <c r="I11" s="36" t="n">
+      <c r="I11" s="36">
         <v>0</v>
       </c>
-      <c r="J11" s="37" t="n">
+      <c r="J11" s="37">
         <v>0</v>
       </c>
-      <c r="K11" s="33" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L11" s="36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M11" s="36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N11" s="36" t="n">
+      <c r="K11" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="L11" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="M11" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="N11" s="36">
         <v>3</v>
       </c>
-      <c r="O11" s="37" t="n">
+      <c r="O11" s="37">
         <v>3</v>
       </c>
     </row>
-    <row r="12" ht="15.6" customHeight="1">
-      <c r="A12" s="1" t="n"/>
-      <c r="B12" s="70" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>FIAS</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="n">
+    <row r="12" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="1"/>
+      <c r="B12" s="70" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="19">
         <v>9.92</v>
       </c>
-      <c r="E12" s="20" t="n">
-        <v>0.9018181818181819</v>
-      </c>
-      <c r="F12" s="21" t="n">
+      <c r="E12" s="20">
+        <v>0.90181818181818185</v>
+      </c>
+      <c r="F12" s="21">
         <v>0</v>
       </c>
-      <c r="G12" s="19" t="n">
+      <c r="G12" s="19">
         <v>5</v>
       </c>
-      <c r="H12" s="22" t="n">
+      <c r="H12" s="22">
         <v>5</v>
       </c>
-      <c r="I12" s="22" t="n">
+      <c r="I12" s="22">
         <v>94</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="J12" s="23">
         <v>109</v>
       </c>
-      <c r="K12" s="19" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L12" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M12" s="22" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N12" s="22" t="n">
+      <c r="K12" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="L12" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="M12" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="N12" s="22">
         <v>0</v>
       </c>
-      <c r="O12" s="23" t="n">
+      <c r="O12" s="23">
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="15.6" customHeight="1">
-      <c r="A13" s="1" t="n"/>
-      <c r="B13" s="67" t="n"/>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>GeYSI</t>
-        </is>
-      </c>
-      <c r="D13" s="25" t="n">
+    <row r="13" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="1"/>
+      <c r="B13" s="67"/>
+      <c r="C13" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="25">
         <v>6.6</v>
       </c>
-      <c r="E13" s="26" t="n">
+      <c r="E13" s="26">
         <v>0.6</v>
       </c>
-      <c r="F13" s="27" t="n">
+      <c r="F13" s="27">
         <v>0</v>
       </c>
-      <c r="G13" s="25" t="n">
+      <c r="G13" s="25">
         <v>4</v>
       </c>
-      <c r="H13" s="28" t="n">
+      <c r="H13" s="28">
         <v>3</v>
       </c>
-      <c r="I13" s="28" t="n">
+      <c r="I13" s="28">
         <v>1912</v>
       </c>
-      <c r="J13" s="29" t="n">
+      <c r="J13" s="29">
         <v>156</v>
       </c>
-      <c r="K13" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L13" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M13" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N13" s="28" t="n">
+      <c r="K13" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L13" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M13" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="N13" s="28">
         <v>0</v>
       </c>
-      <c r="O13" s="29" t="n">
+      <c r="O13" s="29">
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="15.6" customHeight="1">
-      <c r="A14" s="1" t="n"/>
-      <c r="B14" s="67" t="n"/>
-      <c r="C14" s="24" t="inlineStr">
-        <is>
-          <t>RCA</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="n">
+    <row r="14" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="1"/>
+      <c r="B14" s="67"/>
+      <c r="C14" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="25">
         <v>13.33</v>
       </c>
-      <c r="E14" s="26" t="n">
-        <v>2.666</v>
-      </c>
-      <c r="F14" s="27" t="n">
+      <c r="E14" s="26">
+        <v>2.6659999999999999</v>
+      </c>
+      <c r="F14" s="27">
         <v>1</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G14" s="25">
         <v>1</v>
       </c>
-      <c r="H14" s="28" t="n">
+      <c r="H14" s="28">
         <v>2</v>
       </c>
-      <c r="I14" s="28" t="n">
+      <c r="I14" s="28">
         <v>0</v>
       </c>
-      <c r="J14" s="29" t="n">
+      <c r="J14" s="29">
         <v>0</v>
       </c>
-      <c r="K14" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L14" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M14" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N14" s="28" t="n">
+      <c r="K14" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L14" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M14" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="N14" s="28">
         <v>0</v>
       </c>
-      <c r="O14" s="29" t="n">
+      <c r="O14" s="29">
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="15.6" customHeight="1">
-      <c r="A15" s="1" t="n"/>
-      <c r="B15" s="67" t="n"/>
-      <c r="C15" s="24" t="inlineStr">
-        <is>
-          <t>Nutrition</t>
-        </is>
-      </c>
-      <c r="D15" s="25" t="n">
+    <row r="15" spans="1:21" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1"/>
+      <c r="B15" s="67"/>
+      <c r="C15" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="25">
         <v>12.5</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="26">
         <v>3.125</v>
       </c>
-      <c r="F15" s="27" t="n">
+      <c r="F15" s="27">
         <v>0</v>
       </c>
-      <c r="G15" s="25" t="n">
+      <c r="G15" s="25">
         <v>2</v>
       </c>
-      <c r="H15" s="28" t="n">
+      <c r="H15" s="28">
         <v>8</v>
       </c>
-      <c r="I15" s="28" t="n">
+      <c r="I15" s="28">
         <v>130</v>
       </c>
-      <c r="J15" s="29" t="n">
+      <c r="J15" s="29">
         <v>15</v>
       </c>
-      <c r="K15" s="25" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L15" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M15" s="28" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N15" s="28" t="n">
+      <c r="K15" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="M15" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="N15" s="28">
         <v>0</v>
       </c>
-      <c r="O15" s="29" t="n">
+      <c r="O15" s="29">
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="15.6" customHeight="1" thickBot="1">
-      <c r="A16" s="1" t="n"/>
-      <c r="B16" s="71" t="n"/>
-      <c r="C16" s="32" t="inlineStr">
-        <is>
-          <t>VCMA</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="n">
+    <row r="16" spans="1:21" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1"/>
+      <c r="B16" s="71"/>
+      <c r="C16" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="33">
         <v>3</v>
       </c>
-      <c r="E16" s="34" t="n">
+      <c r="E16" s="34">
         <v>0.3</v>
       </c>
-      <c r="F16" s="35" t="n">
+      <c r="F16" s="35">
         <v>0</v>
       </c>
-      <c r="G16" s="33" t="n">
+      <c r="G16" s="33">
         <v>5</v>
       </c>
-      <c r="H16" s="36" t="n">
+      <c r="H16" s="36">
         <v>3</v>
       </c>
-      <c r="I16" s="36" t="n">
+      <c r="I16" s="36">
         <v>1007</v>
       </c>
-      <c r="J16" s="37" t="n">
+      <c r="J16" s="37">
         <v>81</v>
       </c>
-      <c r="K16" s="33" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="L16" s="36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M16" s="36" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N16" s="36" t="n">
+      <c r="K16" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="L16" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="M16" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="N16" s="36">
         <v>5</v>
       </c>
-      <c r="O16" s="37" t="n">
+      <c r="O16" s="37">
         <v>0</v>
       </c>
     </row>
-    <row r="17" customFormat="1" s="44">
-      <c r="A17" s="38" t="n"/>
-      <c r="B17" s="38" t="n"/>
-      <c r="C17" s="39" t="inlineStr">
-        <is>
-          <t>2025 Actual Values</t>
-        </is>
+    <row r="17" spans="1:21" s="44" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="38"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="39" t="s">
+        <v>33</v>
       </c>
       <c r="D17" s="40">
         <f>SUM(D4:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="41" t="n">
+        <v>216.97</v>
+      </c>
+      <c r="E17" s="41">
         <v>1.3</v>
       </c>
       <c r="F17" s="40">
-        <f>SUM(F4:F16)</f>
-        <v/>
+        <f t="shared" ref="F17:K17" si="0">SUM(F4:F16)</f>
+        <v>6</v>
       </c>
       <c r="G17" s="40">
-        <f>SUM(G4:G16)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>113</v>
       </c>
       <c r="H17" s="40">
-        <f>SUM(H4:H16)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>103</v>
       </c>
       <c r="I17" s="40">
-        <f>SUM(I4:I16)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>12612</v>
       </c>
       <c r="J17" s="40">
-        <f>SUM(J4:J16)</f>
-        <v/>
+        <f t="shared" si="0"/>
+        <v>1444</v>
       </c>
       <c r="K17" s="40">
-        <f>SUM(K4:K16)</f>
-        <v/>
-      </c>
-      <c r="L17" s="40" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="M17" s="42" t="n">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="L17" s="40">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="M17" s="42">
         <v>1</v>
       </c>
       <c r="N17" s="40">
         <f>SUM(N4:N16)</f>
-        <v/>
+        <v>51</v>
       </c>
       <c r="O17" s="40">
         <f>SUM(O4:O16)</f>
-        <v/>
-      </c>
-      <c r="P17" s="39" t="n"/>
-      <c r="Q17" s="43" t="n"/>
-      <c r="R17" s="43" t="n"/>
-      <c r="S17" s="43" t="n"/>
-      <c r="T17" s="43" t="n"/>
-      <c r="U17" s="43" t="n"/>
+        <v>23</v>
+      </c>
+      <c r="P17" s="39"/>
+      <c r="Q17" s="43"/>
+      <c r="R17" s="43"/>
+      <c r="S17" s="43"/>
+      <c r="T17" s="43"/>
+      <c r="U17" s="43"/>
     </row>
-    <row r="18" customFormat="1" s="45">
-      <c r="C18" s="46" t="inlineStr">
-        <is>
-          <t>Annual Target</t>
-        </is>
-      </c>
-      <c r="D18" s="46" t="n">
+    <row r="18" spans="1:21" s="45" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="46">
         <v>272</v>
       </c>
-      <c r="E18" s="47" t="n">
+      <c r="E18" s="47">
         <v>2</v>
       </c>
-      <c r="F18" s="48" t="n">
+      <c r="F18" s="48">
         <v>13</v>
       </c>
-      <c r="G18" s="46" t="n">
+      <c r="G18" s="46">
         <v>150</v>
       </c>
-      <c r="H18" s="46" t="n">
+      <c r="H18" s="46">
         <v>60</v>
       </c>
-      <c r="I18" s="49" t="n">
+      <c r="I18" s="49">
         <v>12000</v>
       </c>
-      <c r="J18" s="46" t="n">
+      <c r="J18" s="46">
         <v>150</v>
       </c>
-      <c r="K18" s="46" t="n">
+      <c r="K18" s="46">
         <v>6</v>
       </c>
-      <c r="L18" s="50" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="M18" s="51" t="n">
+      <c r="L18" s="50">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="M18" s="51">
         <v>1</v>
       </c>
-      <c r="N18" s="46" t="n">
+      <c r="N18" s="46">
         <v>20</v>
       </c>
-      <c r="O18" s="46" t="n">
+      <c r="O18" s="46">
         <v>30</v>
       </c>
-      <c r="P18" s="46" t="n"/>
-      <c r="Q18" s="53" t="n"/>
-      <c r="R18" s="53" t="n"/>
-      <c r="S18" s="53" t="n"/>
-      <c r="T18" s="53" t="n"/>
-      <c r="U18" s="53" t="n"/>
+      <c r="P18" s="46"/>
+      <c r="Q18" s="53"/>
+      <c r="R18" s="53"/>
+      <c r="S18" s="53"/>
+      <c r="T18" s="53"/>
+      <c r="U18" s="53"/>
     </row>
-    <row r="19" customFormat="1" s="45">
-      <c r="C19" s="46" t="inlineStr">
-        <is>
-          <t>Per Program Target (target/13)</t>
-        </is>
+    <row r="19" spans="1:21" s="45" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="46" t="s">
+        <v>35</v>
       </c>
       <c r="D19" s="54">
         <f>D18/13</f>
-        <v/>
-      </c>
-      <c r="E19" s="54" t="n">
+        <v>20.923076923076923</v>
+      </c>
+      <c r="E19" s="54">
         <v>2</v>
       </c>
-      <c r="F19" s="54" t="n">
+      <c r="F19" s="54">
         <v>1</v>
       </c>
       <c r="G19" s="54">
         <f>G18/13</f>
-        <v/>
+        <v>11.538461538461538</v>
       </c>
       <c r="H19" s="54">
         <f>H18/13</f>
-        <v/>
+        <v>4.615384615384615</v>
       </c>
       <c r="I19" s="54">
         <f>I18/13</f>
-        <v/>
+        <v>923.07692307692309</v>
       </c>
       <c r="J19" s="54">
         <f>J18/13</f>
-        <v/>
-      </c>
-      <c r="K19" s="54" t="n"/>
-      <c r="L19" s="54" t="n"/>
-      <c r="M19" s="54" t="n"/>
+        <v>11.538461538461538</v>
+      </c>
+      <c r="K19" s="54"/>
+      <c r="L19" s="54"/>
+      <c r="M19" s="54"/>
       <c r="N19" s="54">
         <f>N18/13</f>
-        <v/>
+        <v>1.5384615384615385</v>
       </c>
       <c r="O19" s="54">
         <f>O18/13</f>
-        <v/>
-      </c>
-      <c r="P19" s="52" t="n"/>
-      <c r="Q19" s="53" t="n"/>
-      <c r="R19" s="53" t="n"/>
-      <c r="S19" s="53" t="n"/>
-      <c r="T19" s="53" t="n"/>
-      <c r="U19" s="53" t="n"/>
+        <v>2.3076923076923075</v>
+      </c>
+      <c r="P19" s="52"/>
+      <c r="Q19" s="53"/>
+      <c r="R19" s="53"/>
+      <c r="S19" s="53"/>
+      <c r="T19" s="53"/>
+      <c r="U19" s="53"/>
     </row>
-    <row r="20"/>
-    <row r="21" hidden="1" ht="18" customHeight="1">
-      <c r="C21" s="55" t="n"/>
-      <c r="D21" s="56" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
+    <row r="21" spans="1:21" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C21" s="55"/>
+      <c r="D21" s="56" t="s">
+        <v>36</v>
       </c>
     </row>
-    <row r="22" hidden="1" ht="18" customHeight="1">
-      <c r="D22" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">It looks like the colorscheme is not consistently applied everywhere </t>
-        </is>
+    <row r="22" spans="1:21" ht="18" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D22" s="60" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="23" hidden="1" ht="21" customHeight="1">
-      <c r="D23" s="61" t="inlineStr">
-        <is>
-          <t>(e.g., see the different versions of red in cells G4 and H4)?</t>
-        </is>
+    <row r="23" spans="1:21" ht="21" hidden="1" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="D23" s="61" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="24" hidden="1">
-      <c r="C24" s="62" t="n"/>
+    <row r="24" spans="1:21" hidden="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="C1:O1"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="B4:B7"/>
     <mergeCell ref="K2:O2"/>
     <mergeCell ref="B12:B16"/>
     <mergeCell ref="G2:J2"/>
-    <mergeCell ref="C1:O1"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D16">
     <cfRule type="colorScale" priority="216">
@@ -2184,8 +2118,8 @@
     </cfRule>
     <cfRule type="colorScale" priority="217">
       <colorScale>
-        <cfvo type="formula" val="$E$19"/>
-        <cfvo type="num" val="0"/>
+        <cfvo type="formula" val="&quot;lowest()&quot;"/>
+        <cfvo type="num" val="$E$18/2"/>
         <cfvo type="formula" val="$E$18"/>
         <color rgb="FFFF0000"/>
         <color rgb="FFFFFF00"/>
@@ -2755,7 +2689,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5 M6">
+  <conditionalFormatting sqref="M6 K5">
     <cfRule type="colorScale" priority="112">
       <colorScale>
         <cfvo type="min"/>
@@ -2822,6 +2756,12 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="8" scale="60"/>
+  <pageSetup paperSize="8" scale="60" orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9d258917-277f-42cd-a3cd-14c4e9ee58bc}" enabled="1" method="Standard" siteId="{38ae3bcd-9579-4fd4-adda-b42e1495d55a}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Modified files after review
</commit_message>
<xml_diff>
--- a/data/Heat map 1.xlsx
+++ b/data/Heat map 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EEDDFC8-6033-44A2-823B-3C56C9390FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C91CEC-5FB7-4C82-8F93-BD60EC1D4D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7BB6CA40-8772-4230-BA57-5A736E483AF1}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_Hlk200085589" localSheetId="0">'Res, Cap, Product'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Res, Cap, Product'!$B$1:$P$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Res, Cap, Product'!$B$1:$O$19</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -169,7 +169,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,20 +202,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF0070C0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -701,7 +687,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -723,9 +709,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="1"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -737,15 +720,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
@@ -755,15 +733,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="21" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
@@ -842,37 +820,34 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -881,54 +856,54 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1271,72 +1246,61 @@
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:U24"/>
+  <dimension ref="B1:P24"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="3.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.33203125" style="22" customWidth="1"/>
+    <col min="3" max="3" width="33.33203125" style="18" customWidth="1"/>
     <col min="4" max="4" width="8" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8" style="20" customWidth="1"/>
-    <col min="6" max="6" width="8" style="21" customWidth="1"/>
+    <col min="5" max="5" width="8" style="16" customWidth="1"/>
+    <col min="6" max="6" width="8" style="17" customWidth="1"/>
     <col min="7" max="15" width="8" style="1" customWidth="1"/>
-    <col min="16" max="16" width="4" style="1" customWidth="1"/>
-    <col min="17" max="21" width="8.21875" style="2" customWidth="1"/>
+    <col min="16" max="16" width="8.21875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:21" s="11" customFormat="1" ht="12.6" thickBot="1">
+    <row r="1" spans="2:16" s="10" customFormat="1" ht="12.6" thickBot="1">
       <c r="B1" s="3"/>
-      <c r="C1" s="78" t="s">
+      <c r="C1" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="79"/>
-      <c r="O1" s="80"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="10"/>
-      <c r="R1" s="10"/>
-      <c r="S1" s="10"/>
-      <c r="T1" s="10"/>
-      <c r="U1" s="10"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="N1" s="74"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="9"/>
     </row>
-    <row r="2" spans="2:21" s="66" customFormat="1" ht="12.6" thickBot="1">
-      <c r="B2" s="62"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="81" t="s">
+    <row r="2" spans="2:16" s="61" customFormat="1" ht="12.6" thickBot="1">
+      <c r="B2" s="58"/>
+      <c r="C2" s="59"/>
+      <c r="D2" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="82"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="84" t="s">
+      <c r="E2" s="77"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="86"/>
-      <c r="K2" s="84" t="s">
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="85"/>
-      <c r="M2" s="85"/>
-      <c r="N2" s="85"/>
-      <c r="O2" s="86"/>
-      <c r="P2" s="64"/>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="65"/>
-      <c r="S2" s="65"/>
-      <c r="T2" s="65"/>
-      <c r="U2" s="65"/>
+      <c r="L2" s="80"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="80"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="60"/>
     </row>
-    <row r="3" spans="2:21" s="11" customFormat="1" ht="143.55000000000001" customHeight="1" thickBot="1">
+    <row r="3" spans="2:16" s="10" customFormat="1" ht="143.55000000000001" customHeight="1" thickBot="1">
       <c r="B3" s="3"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5" t="s">
@@ -1376,837 +1340,752 @@
         <v>38</v>
       </c>
       <c r="P3" s="9"/>
-      <c r="Q3" s="10"/>
-      <c r="R3" s="10"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3" s="10"/>
     </row>
-    <row r="4" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B4" s="75" t="s">
+    <row r="4" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B4" s="70" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="31">
+      <c r="D4" s="27">
         <v>21.95</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="28">
         <v>3.1357142857142857</v>
       </c>
-      <c r="F4" s="33">
+      <c r="F4" s="29">
         <v>1</v>
       </c>
-      <c r="G4" s="31">
+      <c r="G4" s="27">
         <v>1</v>
       </c>
-      <c r="H4" s="34">
+      <c r="H4" s="30">
         <v>1</v>
       </c>
-      <c r="I4" s="46">
+      <c r="I4" s="42">
         <v>68</v>
       </c>
-      <c r="J4" s="47">
+      <c r="J4" s="43">
         <v>184</v>
       </c>
-      <c r="K4" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="L4" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="M4" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="N4" s="34">
+      <c r="K4" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="L4" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="M4" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="N4" s="30">
         <v>1</v>
       </c>
-      <c r="O4" s="35">
+      <c r="O4" s="31">
         <v>0</v>
       </c>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
-      <c r="S4" s="10"/>
-      <c r="T4" s="10"/>
-      <c r="U4" s="10"/>
+      <c r="P4" s="9"/>
     </row>
-    <row r="5" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B5" s="76"/>
-      <c r="C5" s="13" t="s">
+    <row r="5" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B5" s="71"/>
+      <c r="C5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="36">
+      <c r="D5" s="32">
         <v>51.45</v>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="33">
         <v>2.2369565217391307</v>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="34">
         <v>0</v>
       </c>
-      <c r="G5" s="36">
+      <c r="G5" s="32">
         <v>24</v>
       </c>
-      <c r="H5" s="39">
+      <c r="H5" s="35">
         <v>28</v>
       </c>
-      <c r="I5" s="48">
+      <c r="I5" s="44">
         <v>108</v>
       </c>
-      <c r="J5" s="49">
+      <c r="J5" s="45">
         <v>214</v>
       </c>
-      <c r="K5" s="36">
+      <c r="K5" s="32">
         <v>15</v>
       </c>
-      <c r="L5" s="26">
+      <c r="L5" s="22">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="M5" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="N5" s="39">
-        <v>8</v>
-      </c>
-      <c r="O5" s="40">
+      <c r="M5" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="N5" s="35">
+        <v>8</v>
+      </c>
+      <c r="O5" s="36">
         <v>5</v>
       </c>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="10"/>
-      <c r="U5" s="10"/>
+      <c r="P5" s="9"/>
     </row>
-    <row r="6" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B6" s="76"/>
-      <c r="C6" s="13" t="s">
+    <row r="6" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B6" s="71"/>
+      <c r="C6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="36">
+      <c r="D6" s="32">
         <v>5</v>
       </c>
-      <c r="E6" s="37">
+      <c r="E6" s="33">
         <v>1.25</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="34">
         <v>0</v>
       </c>
-      <c r="G6" s="36">
+      <c r="G6" s="32">
         <v>26</v>
       </c>
-      <c r="H6" s="39">
+      <c r="H6" s="35">
         <v>19</v>
       </c>
-      <c r="I6" s="48">
+      <c r="I6" s="44">
         <v>5</v>
       </c>
-      <c r="J6" s="49">
+      <c r="J6" s="45">
         <v>113</v>
       </c>
-      <c r="K6" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="L6" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="M6" s="27">
+      <c r="K6" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="L6" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M6" s="23">
         <v>1</v>
       </c>
-      <c r="N6" s="39">
+      <c r="N6" s="35">
         <v>0</v>
       </c>
-      <c r="O6" s="40">
+      <c r="O6" s="36">
         <v>0</v>
       </c>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="10"/>
+      <c r="P6" s="9"/>
     </row>
-    <row r="7" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B7" s="77"/>
-      <c r="C7" s="14" t="s">
+    <row r="7" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
+      <c r="B7" s="72"/>
+      <c r="C7" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="41">
+      <c r="D7" s="37">
         <v>15.4</v>
       </c>
-      <c r="E7" s="42">
+      <c r="E7" s="38">
         <v>1.0266666666666666</v>
       </c>
-      <c r="F7" s="43">
+      <c r="F7" s="39">
         <v>0</v>
       </c>
-      <c r="G7" s="41">
+      <c r="G7" s="37">
         <v>5</v>
       </c>
-      <c r="H7" s="44">
+      <c r="H7" s="40">
         <v>7</v>
       </c>
-      <c r="I7" s="50">
+      <c r="I7" s="46">
         <v>2247</v>
       </c>
-      <c r="J7" s="51">
+      <c r="J7" s="47">
         <v>309</v>
       </c>
-      <c r="K7" s="41" t="s">
-        <v>8</v>
-      </c>
-      <c r="L7" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="M7" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="N7" s="44">
+      <c r="K7" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="L7" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="M7" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="N7" s="40">
         <v>17</v>
       </c>
-      <c r="O7" s="45">
+      <c r="O7" s="41">
         <v>2</v>
       </c>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="10"/>
-      <c r="R7" s="10"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
-      <c r="U7" s="10"/>
+      <c r="P7" s="9"/>
     </row>
-    <row r="8" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B8" s="75" t="s">
+    <row r="8" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B8" s="70" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="27">
         <v>41.45</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="28">
         <v>3.4541666666666671</v>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="29">
         <v>1</v>
       </c>
-      <c r="G8" s="31">
+      <c r="G8" s="27">
         <v>9</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="30">
         <v>9</v>
       </c>
-      <c r="I8" s="46">
+      <c r="I8" s="42">
         <v>102</v>
       </c>
-      <c r="J8" s="47">
+      <c r="J8" s="43">
         <v>10</v>
       </c>
-      <c r="K8" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="L8" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="M8" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="N8" s="34">
+      <c r="K8" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="L8" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="M8" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="N8" s="30">
         <v>6</v>
       </c>
-      <c r="O8" s="35">
+      <c r="O8" s="31">
         <v>2</v>
       </c>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="10"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="10"/>
+      <c r="P8" s="9"/>
     </row>
-    <row r="9" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B9" s="76"/>
-      <c r="C9" s="13" t="s">
+    <row r="9" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B9" s="71"/>
+      <c r="C9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="36">
+      <c r="D9" s="32">
         <v>20.87</v>
       </c>
-      <c r="E9" s="37">
+      <c r="E9" s="33">
         <v>1.0435000000000001</v>
       </c>
-      <c r="F9" s="38">
+      <c r="F9" s="34">
         <v>1</v>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="32">
         <v>22</v>
       </c>
-      <c r="H9" s="39">
+      <c r="H9" s="35">
         <v>14</v>
       </c>
-      <c r="I9" s="48">
+      <c r="I9" s="44">
         <v>3185</v>
       </c>
-      <c r="J9" s="49">
+      <c r="J9" s="45">
         <v>233</v>
       </c>
-      <c r="K9" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="L9" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="M9" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="N9" s="39">
+      <c r="K9" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="L9" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M9" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="N9" s="35">
         <v>1</v>
       </c>
-      <c r="O9" s="40">
+      <c r="O9" s="36">
         <v>9</v>
       </c>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="10"/>
+      <c r="P9" s="9"/>
     </row>
-    <row r="10" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B10" s="76"/>
-      <c r="C10" s="13" t="s">
+    <row r="10" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B10" s="71"/>
+      <c r="C10" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="36">
+      <c r="D10" s="32">
         <v>15.5</v>
       </c>
-      <c r="E10" s="37">
+      <c r="E10" s="33">
         <v>2.2142857142857144</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="34">
         <v>2</v>
       </c>
-      <c r="G10" s="36">
+      <c r="G10" s="32">
         <v>7</v>
       </c>
-      <c r="H10" s="39">
+      <c r="H10" s="35">
         <v>3</v>
       </c>
-      <c r="I10" s="48">
+      <c r="I10" s="44">
         <v>3754</v>
       </c>
-      <c r="J10" s="49">
+      <c r="J10" s="45">
         <v>20</v>
       </c>
-      <c r="K10" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="L10" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="M10" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="N10" s="39">
+      <c r="K10" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="L10" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M10" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="N10" s="35">
         <v>10</v>
       </c>
-      <c r="O10" s="40">
+      <c r="O10" s="36">
         <v>2</v>
       </c>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="10"/>
+      <c r="P10" s="9"/>
     </row>
-    <row r="11" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
-      <c r="B11" s="77"/>
-      <c r="C11" s="14" t="s">
+    <row r="11" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
+      <c r="B11" s="72"/>
+      <c r="C11" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="41">
+      <c r="D11" s="37">
         <v>0</v>
       </c>
-      <c r="E11" s="42">
+      <c r="E11" s="38">
         <v>0</v>
       </c>
-      <c r="F11" s="43">
+      <c r="F11" s="39">
         <v>0</v>
       </c>
-      <c r="G11" s="41">
+      <c r="G11" s="37">
         <v>2</v>
       </c>
-      <c r="H11" s="44">
+      <c r="H11" s="40">
         <v>1</v>
       </c>
-      <c r="I11" s="50">
+      <c r="I11" s="46">
         <v>0</v>
       </c>
-      <c r="J11" s="51">
+      <c r="J11" s="47">
         <v>0</v>
       </c>
-      <c r="K11" s="41" t="s">
-        <v>8</v>
-      </c>
-      <c r="L11" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="M11" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="N11" s="44">
+      <c r="K11" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="L11" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="M11" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="N11" s="40">
         <v>3</v>
       </c>
-      <c r="O11" s="45">
+      <c r="O11" s="41">
         <v>3</v>
       </c>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="10"/>
-      <c r="S11" s="10"/>
-      <c r="T11" s="10"/>
-      <c r="U11" s="10"/>
+      <c r="P11" s="9"/>
     </row>
-    <row r="12" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B12" s="72" t="s">
+    <row r="12" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B12" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="31">
+      <c r="D12" s="27">
         <v>9.92</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="28">
         <v>0.90181818181818185</v>
       </c>
-      <c r="F12" s="33">
+      <c r="F12" s="29">
         <v>0</v>
       </c>
-      <c r="G12" s="31">
+      <c r="G12" s="27">
         <v>5</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="30">
         <v>5</v>
       </c>
-      <c r="I12" s="46">
+      <c r="I12" s="42">
         <v>94</v>
       </c>
-      <c r="J12" s="47">
+      <c r="J12" s="43">
         <v>109</v>
       </c>
-      <c r="K12" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="L12" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="M12" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="N12" s="34">
+      <c r="K12" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="L12" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="M12" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="N12" s="30">
         <v>0</v>
       </c>
-      <c r="O12" s="35">
+      <c r="O12" s="31">
         <v>0</v>
       </c>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="10"/>
-      <c r="R12" s="10"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="10"/>
-      <c r="U12" s="10"/>
+      <c r="P12" s="9"/>
     </row>
-    <row r="13" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B13" s="73"/>
-      <c r="C13" s="13" t="s">
+    <row r="13" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B13" s="68"/>
+      <c r="C13" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="36">
+      <c r="D13" s="32">
         <v>6.6</v>
       </c>
-      <c r="E13" s="37">
+      <c r="E13" s="33">
         <v>0.6</v>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="34">
         <v>0</v>
       </c>
-      <c r="G13" s="36">
+      <c r="G13" s="32">
         <v>4</v>
       </c>
-      <c r="H13" s="39">
+      <c r="H13" s="35">
         <v>3</v>
       </c>
-      <c r="I13" s="48">
+      <c r="I13" s="44">
         <v>1912</v>
       </c>
-      <c r="J13" s="49">
+      <c r="J13" s="45">
         <v>156</v>
       </c>
-      <c r="K13" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="L13" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="M13" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="N13" s="39">
+      <c r="K13" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="L13" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M13" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="N13" s="35">
         <v>0</v>
       </c>
-      <c r="O13" s="40">
+      <c r="O13" s="36">
         <v>0</v>
       </c>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="10"/>
-      <c r="R13" s="10"/>
-      <c r="S13" s="10"/>
-      <c r="T13" s="10"/>
-      <c r="U13" s="10"/>
+      <c r="P13" s="9"/>
     </row>
-    <row r="14" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B14" s="73"/>
-      <c r="C14" s="13" t="s">
+    <row r="14" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B14" s="68"/>
+      <c r="C14" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="36">
+      <c r="D14" s="32">
         <v>13.33</v>
       </c>
-      <c r="E14" s="37">
+      <c r="E14" s="33">
         <v>2.6659999999999999</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="34">
         <v>1</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="32">
         <v>1</v>
       </c>
-      <c r="H14" s="39">
+      <c r="H14" s="35">
         <v>2</v>
       </c>
-      <c r="I14" s="48">
+      <c r="I14" s="44">
         <v>0</v>
       </c>
-      <c r="J14" s="49">
+      <c r="J14" s="45">
         <v>0</v>
       </c>
-      <c r="K14" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="L14" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="M14" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="N14" s="39">
+      <c r="K14" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="L14" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M14" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="N14" s="35">
         <v>0</v>
       </c>
-      <c r="O14" s="40">
+      <c r="O14" s="36">
         <v>0</v>
       </c>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="10"/>
-      <c r="R14" s="10"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
-      <c r="U14" s="10"/>
+      <c r="P14" s="9"/>
     </row>
-    <row r="15" spans="2:21" s="11" customFormat="1" ht="15.6" customHeight="1">
-      <c r="B15" s="73"/>
-      <c r="C15" s="13" t="s">
+    <row r="15" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+      <c r="B15" s="68"/>
+      <c r="C15" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="36">
+      <c r="D15" s="32">
         <v>12.5</v>
       </c>
-      <c r="E15" s="37">
+      <c r="E15" s="33">
         <v>3.125</v>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="34">
         <v>0</v>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="32">
         <v>2</v>
       </c>
-      <c r="H15" s="39">
-        <v>8</v>
-      </c>
-      <c r="I15" s="48">
+      <c r="H15" s="35">
+        <v>8</v>
+      </c>
+      <c r="I15" s="44">
         <v>130</v>
       </c>
-      <c r="J15" s="49">
+      <c r="J15" s="45">
         <v>15</v>
       </c>
-      <c r="K15" s="36" t="s">
-        <v>8</v>
-      </c>
-      <c r="L15" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="M15" s="39" t="s">
-        <v>8</v>
-      </c>
-      <c r="N15" s="39">
+      <c r="K15" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="L15" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="M15" s="35" t="s">
+        <v>8</v>
+      </c>
+      <c r="N15" s="35">
         <v>0</v>
       </c>
-      <c r="O15" s="40">
+      <c r="O15" s="36">
         <v>0</v>
       </c>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="10"/>
-      <c r="R15" s="10"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="10"/>
-      <c r="U15" s="10"/>
+      <c r="P15" s="9"/>
     </row>
-    <row r="16" spans="2:21" s="11" customFormat="1" ht="15.45" customHeight="1" thickBot="1">
-      <c r="B16" s="74"/>
-      <c r="C16" s="14" t="s">
+    <row r="16" spans="2:16" s="10" customFormat="1" ht="15.45" customHeight="1" thickBot="1">
+      <c r="B16" s="69"/>
+      <c r="C16" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="41">
+      <c r="D16" s="37">
         <v>3</v>
       </c>
-      <c r="E16" s="42">
+      <c r="E16" s="38">
         <v>0.3</v>
       </c>
-      <c r="F16" s="43">
+      <c r="F16" s="39">
         <v>0</v>
       </c>
-      <c r="G16" s="41">
+      <c r="G16" s="37">
         <v>5</v>
       </c>
-      <c r="H16" s="44">
+      <c r="H16" s="40">
         <v>3</v>
       </c>
-      <c r="I16" s="50">
+      <c r="I16" s="46">
         <v>1007</v>
       </c>
-      <c r="J16" s="51">
+      <c r="J16" s="47">
         <v>81</v>
       </c>
-      <c r="K16" s="41" t="s">
-        <v>8</v>
-      </c>
-      <c r="L16" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="M16" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="N16" s="44">
+      <c r="K16" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="M16" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="N16" s="40">
         <v>5</v>
       </c>
-      <c r="O16" s="45">
+      <c r="O16" s="41">
         <v>0</v>
       </c>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="10"/>
-      <c r="R16" s="10"/>
-      <c r="S16" s="10"/>
-      <c r="T16" s="10"/>
-      <c r="U16" s="10"/>
+      <c r="P16" s="9"/>
     </row>
-    <row r="17" spans="2:21" s="69" customFormat="1" ht="12">
-      <c r="B17" s="67"/>
-      <c r="C17" s="53" t="s">
+    <row r="17" spans="2:16" s="64" customFormat="1" ht="12">
+      <c r="B17" s="62"/>
+      <c r="C17" s="49" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="54">
+      <c r="D17" s="50">
         <v>272</v>
       </c>
-      <c r="E17" s="55">
+      <c r="E17" s="51">
         <v>2</v>
       </c>
-      <c r="F17" s="56">
+      <c r="F17" s="52">
         <v>13</v>
       </c>
-      <c r="G17" s="54">
+      <c r="G17" s="50">
         <v>150</v>
       </c>
-      <c r="H17" s="54">
+      <c r="H17" s="50">
         <v>60</v>
       </c>
-      <c r="I17" s="57">
+      <c r="I17" s="53">
         <v>12000</v>
       </c>
-      <c r="J17" s="57">
+      <c r="J17" s="53">
         <v>150</v>
       </c>
-      <c r="K17" s="54">
+      <c r="K17" s="50">
         <v>6</v>
       </c>
-      <c r="L17" s="56">
+      <c r="L17" s="52">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="M17" s="54">
+      <c r="M17" s="50">
         <v>1</v>
       </c>
-      <c r="N17" s="54">
+      <c r="N17" s="50">
         <v>20</v>
       </c>
-      <c r="O17" s="54">
+      <c r="O17" s="50">
         <v>30</v>
       </c>
-      <c r="P17" s="16"/>
-      <c r="Q17" s="68"/>
-      <c r="R17" s="68"/>
-      <c r="S17" s="68"/>
-      <c r="T17" s="68"/>
-      <c r="U17" s="68"/>
+      <c r="P17" s="63"/>
     </row>
-    <row r="18" spans="2:21" s="71" customFormat="1" ht="12">
-      <c r="B18" s="52"/>
-      <c r="C18" s="53" t="s">
+    <row r="18" spans="2:16" s="66" customFormat="1" ht="12">
+      <c r="B18" s="48"/>
+      <c r="C18" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="D18" s="58">
+      <c r="D18" s="54">
         <f>SUM(D4:D16)</f>
         <v>216.97</v>
       </c>
-      <c r="E18" s="59">
+      <c r="E18" s="55">
         <f>AVERAGE(E4:E16)</f>
         <v>1.6887775412992805</v>
       </c>
-      <c r="F18" s="55">
+      <c r="F18" s="51">
         <f t="shared" ref="F18:O18" si="0">SUM(F4:F16)</f>
         <v>6</v>
       </c>
-      <c r="G18" s="55">
+      <c r="G18" s="51">
         <f t="shared" si="0"/>
         <v>113</v>
       </c>
-      <c r="H18" s="55">
+      <c r="H18" s="51">
         <f t="shared" si="0"/>
         <v>103</v>
       </c>
-      <c r="I18" s="57">
+      <c r="I18" s="53">
         <f t="shared" si="0"/>
         <v>12612</v>
       </c>
-      <c r="J18" s="57">
+      <c r="J18" s="53">
         <f t="shared" si="0"/>
         <v>1444</v>
       </c>
-      <c r="K18" s="55">
+      <c r="K18" s="51">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="L18" s="60">
+      <c r="L18" s="56">
         <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="M18" s="61">
+      <c r="M18" s="57">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="N18" s="55">
+      <c r="N18" s="51">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
-      <c r="O18" s="55">
+      <c r="O18" s="51">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="70"/>
-      <c r="R18" s="70"/>
-      <c r="S18" s="70"/>
-      <c r="T18" s="70"/>
-      <c r="U18" s="70"/>
+      <c r="P18" s="65"/>
     </row>
-    <row r="19" spans="2:21" s="69" customFormat="1" ht="12">
-      <c r="B19" s="67"/>
-      <c r="C19" s="53" t="s">
+    <row r="19" spans="2:16" s="64" customFormat="1" ht="12">
+      <c r="B19" s="62"/>
+      <c r="C19" s="49" t="s">
         <v>22</v>
       </c>
-      <c r="D19" s="54">
+      <c r="D19" s="50">
         <f>D17/13</f>
         <v>20.923076923076923</v>
       </c>
-      <c r="E19" s="54">
+      <c r="E19" s="50">
         <v>2</v>
       </c>
-      <c r="F19" s="54">
+      <c r="F19" s="50">
         <v>1</v>
       </c>
-      <c r="G19" s="54">
+      <c r="G19" s="50">
         <f>G17/13</f>
         <v>11.538461538461538</v>
       </c>
-      <c r="H19" s="54">
+      <c r="H19" s="50">
         <f>H17/13</f>
         <v>4.615384615384615</v>
       </c>
-      <c r="I19" s="57">
+      <c r="I19" s="53">
         <f>I17/13</f>
         <v>923.07692307692309</v>
       </c>
-      <c r="J19" s="57">
+      <c r="J19" s="53">
         <f>J17/13</f>
         <v>11.538461538461538</v>
       </c>
-      <c r="K19" s="54" t="s">
-        <v>8</v>
-      </c>
-      <c r="L19" s="54" t="s">
-        <v>8</v>
-      </c>
-      <c r="M19" s="54" t="s">
-        <v>8</v>
-      </c>
-      <c r="N19" s="54">
+      <c r="K19" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="L19" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="M19" s="50" t="s">
+        <v>8</v>
+      </c>
+      <c r="N19" s="50">
         <f>N17/13</f>
         <v>1.5384615384615385</v>
       </c>
-      <c r="O19" s="54">
+      <c r="O19" s="50">
         <f>O17/13</f>
         <v>2.3076923076923075</v>
       </c>
-      <c r="P19" s="17"/>
-      <c r="Q19" s="68"/>
-      <c r="R19" s="68"/>
-      <c r="S19" s="68"/>
-      <c r="T19" s="68"/>
-      <c r="U19" s="68"/>
+      <c r="P19" s="63"/>
     </row>
-    <row r="20" spans="2:21">
-      <c r="D20" s="28"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
+    <row r="20" spans="2:16">
+      <c r="D20" s="24"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+      <c r="K20" s="24"/>
+      <c r="L20" s="24"/>
+      <c r="M20" s="24"/>
+      <c r="N20" s="24"/>
+      <c r="O20" s="24"/>
     </row>
-    <row r="21" spans="2:21" ht="18" hidden="1">
-      <c r="C21" s="18"/>
-      <c r="D21" s="19" t="s">
+    <row r="21" spans="2:16" ht="18" hidden="1">
+      <c r="C21" s="14"/>
+      <c r="D21" s="15" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="2:21" ht="18" hidden="1">
-      <c r="D22" s="23" t="s">
+    <row r="22" spans="2:16" ht="18" hidden="1">
+      <c r="D22" s="19" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="2:21" ht="21" hidden="1">
-      <c r="D23" s="24" t="s">
+    <row r="23" spans="2:16" ht="21" hidden="1">
+      <c r="D23" s="20" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="2:21" hidden="1">
-      <c r="C24" s="25"/>
+    <row r="24" spans="2:16" hidden="1">
+      <c r="C24" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2322,38 +2201,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5 M6">
-    <cfRule type="colorScale" priority="107">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="108">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="112">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="K6:L6">
     <cfRule type="colorScale" priority="172">
       <colorScale>
@@ -2833,6 +2680,38 @@
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M6 K5">
+    <cfRule type="colorScale" priority="107">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="108">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="112">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Updated file as per review
</commit_message>
<xml_diff>
--- a/data/Heat map 1.xlsx
+++ b/data/Heat map 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learning\Miscellaneous\KPIDashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C91CEC-5FB7-4C82-8F93-BD60EC1D4D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637945C4-9048-442B-8CCE-19BFFBA0E2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{7BB6CA40-8772-4230-BA57-5A736E483AF1}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7BB6CA40-8772-4230-BA57-5A736E483AF1}"/>
   </bookViews>
   <sheets>
     <sheet name="Res, Cap, Product" sheetId="1" r:id="rId1"/>
@@ -60,9 +60,6 @@
     <t>Annual rate of genetic gain, by crop (%)</t>
   </si>
   <si>
-    <t>GI</t>
-  </si>
-  <si>
     <t>Biotech</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
     <t>Seed System</t>
   </si>
   <si>
-    <t>RAFS</t>
-  </si>
-  <si>
     <t>Plant Health</t>
   </si>
   <si>
@@ -90,9 +84,6 @@
     <t>Mechanization</t>
   </si>
   <si>
-    <t>ST</t>
-  </si>
-  <si>
     <t>2025 Actual Values</t>
   </si>
   <si>
@@ -157,6 +148,15 @@
   </si>
   <si>
     <t>Innovations taken on by scaling partners</t>
+  </si>
+  <si>
+    <t>Genetic Innovation</t>
+  </si>
+  <si>
+    <t>Resilient Agrifood Systems</t>
+  </si>
+  <si>
+    <t>Systems Transformation</t>
   </si>
 </sst>
 </file>
@@ -169,7 +169,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1247,7 +1247,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:P24"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="3.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.33203125" style="18" customWidth="1"/>
@@ -1258,7 +1258,7 @@
     <col min="16" max="16" width="8.21875" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" s="10" customFormat="1" ht="12.6" thickBot="1">
+    <row r="1" spans="2:16" s="10" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="3"/>
       <c r="C1" s="73" t="s">
         <v>0</v>
@@ -1277,7 +1277,7 @@
       <c r="O1" s="75"/>
       <c r="P1" s="9"/>
     </row>
-    <row r="2" spans="2:16" s="61" customFormat="1" ht="12.6" thickBot="1">
+    <row r="2" spans="2:16" s="61" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="58"/>
       <c r="C2" s="59"/>
       <c r="D2" s="76" t="s">
@@ -1300,29 +1300,29 @@
       <c r="O2" s="81"/>
       <c r="P2" s="60"/>
     </row>
-    <row r="3" spans="2:16" s="10" customFormat="1" ht="143.55000000000001" customHeight="1" thickBot="1">
+    <row r="3" spans="2:16" s="10" customFormat="1" ht="143.55000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3"/>
       <c r="C3" s="4"/>
       <c r="D3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>32</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="7" t="s">
-        <v>35</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>4</v>
@@ -1331,22 +1331,22 @@
         <v>5</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="P3" s="9"/>
     </row>
-    <row r="4" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="4" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="70" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>6</v>
-      </c>
-      <c r="C4" s="11" t="s">
-        <v>7</v>
       </c>
       <c r="D4" s="27">
         <v>21.95</v>
@@ -1370,13 +1370,13 @@
         <v>184</v>
       </c>
       <c r="K4" s="27" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L4" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M4" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N4" s="30">
         <v>1</v>
@@ -1386,10 +1386,10 @@
       </c>
       <c r="P4" s="9"/>
     </row>
-    <row r="5" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="5" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="71"/>
       <c r="C5" s="12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="32">
         <v>51.45</v>
@@ -1419,7 +1419,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="M5" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N5" s="35">
         <v>8</v>
@@ -1429,10 +1429,10 @@
       </c>
       <c r="P5" s="9"/>
     </row>
-    <row r="6" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="6" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="71"/>
       <c r="C6" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="32">
         <v>5</v>
@@ -1456,10 +1456,10 @@
         <v>113</v>
       </c>
       <c r="K6" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L6" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M6" s="23">
         <v>1</v>
@@ -1472,10 +1472,10 @@
       </c>
       <c r="P6" s="9"/>
     </row>
-    <row r="7" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
+    <row r="7" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="72"/>
       <c r="C7" s="13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="37">
         <v>15.4</v>
@@ -1499,13 +1499,13 @@
         <v>309</v>
       </c>
       <c r="K7" s="37" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L7" s="40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M7" s="40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N7" s="40">
         <v>17</v>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="P7" s="9"/>
     </row>
-    <row r="8" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="8" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="70" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D8" s="27">
         <v>41.45</v>
@@ -1544,13 +1544,13 @@
         <v>10</v>
       </c>
       <c r="K8" s="27" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L8" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M8" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N8" s="30">
         <v>6</v>
@@ -1560,10 +1560,10 @@
       </c>
       <c r="P8" s="9"/>
     </row>
-    <row r="9" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="9" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="71"/>
       <c r="C9" s="12" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" s="32">
         <v>20.87</v>
@@ -1587,13 +1587,13 @@
         <v>233</v>
       </c>
       <c r="K9" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L9" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M9" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N9" s="35">
         <v>1</v>
@@ -1603,10 +1603,10 @@
       </c>
       <c r="P9" s="9"/>
     </row>
-    <row r="10" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="10" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="71"/>
       <c r="C10" s="12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D10" s="32">
         <v>15.5</v>
@@ -1630,13 +1630,13 @@
         <v>20</v>
       </c>
       <c r="K10" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L10" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M10" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N10" s="35">
         <v>10</v>
@@ -1646,10 +1646,10 @@
       </c>
       <c r="P10" s="9"/>
     </row>
-    <row r="11" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" thickBot="1">
+    <row r="11" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="72"/>
       <c r="C11" s="13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11" s="37">
         <v>0</v>
@@ -1673,13 +1673,13 @@
         <v>0</v>
       </c>
       <c r="K11" s="37" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L11" s="40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M11" s="40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N11" s="40">
         <v>3</v>
@@ -1689,12 +1689,12 @@
       </c>
       <c r="P11" s="9"/>
     </row>
-    <row r="12" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="12" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="67" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D12" s="27">
         <v>9.92</v>
@@ -1718,13 +1718,13 @@
         <v>109</v>
       </c>
       <c r="K12" s="27" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L12" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M12" s="30" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N12" s="30">
         <v>0</v>
@@ -1734,10 +1734,10 @@
       </c>
       <c r="P12" s="9"/>
     </row>
-    <row r="13" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="13" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="68"/>
       <c r="C13" s="12" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D13" s="32">
         <v>6.6</v>
@@ -1761,13 +1761,13 @@
         <v>156</v>
       </c>
       <c r="K13" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L13" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M13" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N13" s="35">
         <v>0</v>
@@ -1777,10 +1777,10 @@
       </c>
       <c r="P13" s="9"/>
     </row>
-    <row r="14" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="14" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="68"/>
       <c r="C14" s="12" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D14" s="32">
         <v>13.33</v>
@@ -1804,13 +1804,13 @@
         <v>0</v>
       </c>
       <c r="K14" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L14" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M14" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N14" s="35">
         <v>0</v>
@@ -1820,10 +1820,10 @@
       </c>
       <c r="P14" s="9"/>
     </row>
-    <row r="15" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1">
+    <row r="15" spans="2:16" s="10" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="68"/>
       <c r="C15" s="12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D15" s="32">
         <v>12.5</v>
@@ -1847,13 +1847,13 @@
         <v>15</v>
       </c>
       <c r="K15" s="32" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L15" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M15" s="35" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N15" s="35">
         <v>0</v>
@@ -1863,10 +1863,10 @@
       </c>
       <c r="P15" s="9"/>
     </row>
-    <row r="16" spans="2:16" s="10" customFormat="1" ht="15.45" customHeight="1" thickBot="1">
+    <row r="16" spans="2:16" s="10" customFormat="1" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="69"/>
       <c r="C16" s="13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D16" s="37">
         <v>3</v>
@@ -1890,13 +1890,13 @@
         <v>81</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L16" s="40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N16" s="40">
         <v>5</v>
@@ -1906,10 +1906,10 @@
       </c>
       <c r="P16" s="9"/>
     </row>
-    <row r="17" spans="2:16" s="64" customFormat="1" ht="12">
+    <row r="17" spans="2:16" s="64" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="B17" s="62"/>
       <c r="C17" s="49" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D17" s="50">
         <v>272</v>
@@ -1949,10 +1949,10 @@
       </c>
       <c r="P17" s="63"/>
     </row>
-    <row r="18" spans="2:16" s="66" customFormat="1" ht="12">
+    <row r="18" spans="2:16" s="66" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="B18" s="48"/>
       <c r="C18" s="49" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D18" s="54">
         <f>SUM(D4:D16)</f>
@@ -2004,10 +2004,10 @@
       </c>
       <c r="P18" s="65"/>
     </row>
-    <row r="19" spans="2:16" s="64" customFormat="1" ht="12">
+    <row r="19" spans="2:16" s="64" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="B19" s="62"/>
       <c r="C19" s="49" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D19" s="50">
         <f>D17/13</f>
@@ -2036,13 +2036,13 @@
         <v>11.538461538461538</v>
       </c>
       <c r="K19" s="50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L19" s="50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M19" s="50" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N19" s="50">
         <f>N17/13</f>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="P19" s="63"/>
     </row>
-    <row r="20" spans="2:16">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.3">
       <c r="D20" s="24"/>
       <c r="E20" s="25"/>
       <c r="F20" s="26"/>
@@ -2068,23 +2068,23 @@
       <c r="N20" s="24"/>
       <c r="O20" s="24"/>
     </row>
-    <row r="21" spans="2:16" ht="18" hidden="1">
+    <row r="21" spans="2:16" ht="18" hidden="1" x14ac:dyDescent="0.35">
       <c r="C21" s="14"/>
       <c r="D21" s="15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="22" spans="2:16" ht="18" hidden="1">
+    <row r="22" spans="2:16" ht="18" hidden="1" x14ac:dyDescent="0.35">
       <c r="D22" s="19" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="23" spans="2:16" ht="21" hidden="1">
+    <row r="23" spans="2:16" ht="21" hidden="1" x14ac:dyDescent="0.4">
       <c r="D23" s="20" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="24" spans="2:16" hidden="1">
+    <row r="24" spans="2:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="C24" s="21"/>
     </row>
   </sheetData>
@@ -2144,6 +2144,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:G16">
+    <cfRule type="colorScale" priority="238">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="237">
       <colorScale>
         <cfvo type="min"/>
@@ -2154,16 +2164,6 @@
         <color rgb="FF00B050"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="238">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H16">
     <cfRule type="colorScale" priority="239">
@@ -2201,17 +2201,39 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="K5 M6">
+    <cfRule type="colorScale" priority="107">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="108">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="112">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K6:L6">
-    <cfRule type="colorScale" priority="172">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="173">
       <colorScale>
         <cfvo type="min"/>
@@ -2222,27 +2244,17 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="174">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="175">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="176">
+    <cfRule type="colorScale" priority="181">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="182">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2252,57 +2264,37 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="177">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="178">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="179">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="180">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="181">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="182">
+    <cfRule type="colorScale" priority="172">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="174">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="175">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="176">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2310,6 +2302,46 @@
         <color rgb="FF63BE7B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="177">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="178">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="179">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="180">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -2374,46 +2406,6 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="189">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="190">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="191">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="192">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="193">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -2424,8 +2416,138 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
+    <cfRule type="colorScale" priority="192">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="191">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="190">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="189">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7:M16">
+    <cfRule type="colorScale" priority="198">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="199">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="200">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="201">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="202">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="203">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="204">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="196">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="195">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="194">
       <colorScale>
         <cfvo type="min"/>
@@ -2436,26 +2558,6 @@
         <color rgb="FFFFFF00"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="195">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="196">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="197">
       <colorScale>
         <cfvo type="min"/>
@@ -2464,76 +2566,6 @@
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="198">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="199">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="200">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="201">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="202">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="203">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="204">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -2572,47 +2604,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M5">
-    <cfRule type="colorScale" priority="205">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="206">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="207">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="208">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="209">
+    <cfRule type="colorScale" priority="214">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="215">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2622,57 +2624,37 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="210">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="211">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="formula" val="MAX(#REF!)/2"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="212">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="213">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="214">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="215">
+    <cfRule type="colorScale" priority="206">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="207">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="208">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="209">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="0"/>
@@ -2682,9 +2664,37 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M6 K5">
-    <cfRule type="colorScale" priority="107">
+    <cfRule type="colorScale" priority="210">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="211">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="MAX(#REF!)/2"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="212">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="205">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="formula" val="MAX($K$4:$K$16)/2"/>
@@ -2694,17 +2704,7 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="108">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="112">
+    <cfRule type="colorScale" priority="213">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2716,6 +2716,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:N16">
+    <cfRule type="colorScale" priority="243">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="242">
       <colorScale>
         <cfvo type="min"/>
@@ -2724,16 +2734,6 @@
         <color rgb="FFFF0000"/>
         <color rgb="FFFFFF00"/>
         <color rgb="FF00B050"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="243">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>